<commit_message>
Split frame pricing by print size
</commit_message>
<xml_diff>
--- a/apps/moment-booth-fe/data/frame-package-pricing.xlsx
+++ b/apps/moment-booth-fe/data/frame-package-pricing.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Frame Pricing" sheetId="1" r:id="R22c6605b6f8041b9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Frame Pricing" sheetId="1" r:id="Rf50c52770c34492d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -18,7 +18,7 @@
     <x:numFmt numFmtId="201" formatCode="0"/>
     <x:numFmt numFmtId="202" formatCode="&quot;$&quot;#,##0.00"/>
   </x:numFmts>
-  <x:fonts count="12">
+  <x:fonts count="14">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -87,8 +87,20 @@
       <x:color rgb="FF6B7280"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="10"/>
+      <x:color rgb="FF6B7280"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="9"/>
+      <x:color rgb="FF6B7280"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="10">
+  <x:fills count="12">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -135,6 +147,16 @@
         <x:fgColor rgb="FFE9DDFF"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE9DDFF"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border>
@@ -148,7 +170,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="47">
+  <x:cellXfs count="58">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -260,6 +282,33 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="10" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="5" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="4" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="7" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -504,7 +553,7 @@
       <x:c r="F2" s="8"/>
       <x:c r="G2" s="8"/>
       <x:c r="H2" s="8" t="str">
-        <x:v>Fill in the yellow Unit Price cells. Original package prices calculate automatically from total frames × unit price; update New Package Price separately.</x:v>
+        <x:v>Fill in the yellow unit-price cells for each size. Original package prices calculate automatically from the size quantities and unit prices; update New Package Price separately.</x:v>
       </x:c>
       <x:c r="I2" s="8"/>
       <x:c r="J2" s="8"/>
@@ -531,28 +580,37 @@
       <x:c r="G4" s="13" t="str">
         <x:v>Material</x:v>
       </x:c>
-      <x:c r="H4" s="44" t="str">
-        <x:v>Unit Price (SGD)</x:v>
-      </x:c>
-      <x:c r="I4" s="44" t="str">
+      <x:c r="H4" s="53" t="str">
+        <x:v>8" Unit Price (SGD)</x:v>
+      </x:c>
+      <x:c r="I4" s="53" t="str">
+        <x:v>10" Unit Price (SGD)</x:v>
+      </x:c>
+      <x:c r="J4" s="53" t="str">
+        <x:v>12" Unit Price (SGD)</x:v>
+      </x:c>
+      <x:c r="K4" s="54" t="str">
         <x:v>Original Price (SGD)</x:v>
       </x:c>
-      <x:c r="J4" s="44" t="str">
+      <x:c r="L4" s="53" t="str">
         <x:v>New Package Price (SGD)</x:v>
       </x:c>
-      <x:c r="K4" s="45" t="str">
+      <x:c r="M4" s="53" t="str">
         <x:v>Notes</x:v>
-      </x:c>
-      <x:c r="L4" s="28" t="str">
-        <x:v>Package guide</x:v>
-      </x:c>
-      <x:c r="M4" s="28" t="str">
-        <x:v>Total frames</x:v>
       </x:c>
       <x:c r="N4" s="28" t="str">
         <x:v>Size breakdown</x:v>
       </x:c>
       <x:c r="O4" s="28" t="str">
+        <x:v>Package guide</x:v>
+      </x:c>
+      <x:c r="P4" t="str">
+        <x:v>Total frames</x:v>
+      </x:c>
+      <x:c r="Q4" t="str">
+        <x:v>Size breakdown</x:v>
+      </x:c>
+      <x:c r="R4" t="str">
         <x:v>Positioning</x:v>
       </x:c>
     </x:row>
@@ -578,26 +636,31 @@
       <x:c r="G5" s="15" t="str">
         <x:v>Frameless Rounded Corner</x:v>
       </x:c>
-      <x:c r="H5" s="39"/>
-      <x:c r="I5" s="40" t="str">
-        <x:f>IF(H5="","",F5*H5)</x:f>
-      </x:c>
-      <x:c r="J5" s="41" t="n">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="K5" s="46" t="str">
-        <x:v>Enter the per-frame unit price in column H.</x:v>
-      </x:c>
-      <x:c r="L5" s="32" t="str">
-        <x:v>6-piece package</x:v>
-      </x:c>
-      <x:c r="M5" s="32" t="n">
-        <x:v>6</x:v>
+      <x:c r="H5" s="47"/>
+      <x:c r="I5" s="47"/>
+      <x:c r="J5" s="48"/>
+      <x:c r="K5" s="49" t="str">
+        <x:f>IF(COUNTA(H5:J5)=0,"",C5*H5+D5*I5+E5*J5)</x:f>
+      </x:c>
+      <x:c r="L5" s="50" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="M5" s="56" t="str">
+        <x:v>Enter the unit prices for 8", 10" and 12" in columns H–J.</x:v>
       </x:c>
       <x:c r="N5" s="32" t="str">
         <x:v>2 × 8", 2 × 10", 2 × 12"</x:v>
       </x:c>
       <x:c r="O5" s="32" t="str">
+        <x:v>6-piece package</x:v>
+      </x:c>
+      <x:c r="P5" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="Q5" t="str">
+        <x:v>2 × 8", 2 × 10", 2 × 12"</x:v>
+      </x:c>
+      <x:c r="R5" t="str">
         <x:v>Standard</x:v>
       </x:c>
     </x:row>
@@ -623,26 +686,31 @@
       <x:c r="G6" s="15" t="str">
         <x:v>White Rounded Border</x:v>
       </x:c>
-      <x:c r="H6" s="39"/>
-      <x:c r="I6" s="40" t="str">
-        <x:f>IF(H6="","",F6*H6)</x:f>
-      </x:c>
-      <x:c r="J6" s="41" t="n">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="K6" s="46" t="str">
-        <x:v>Enter the per-frame unit price in column H.</x:v>
-      </x:c>
-      <x:c r="L6" s="32" t="str">
-        <x:v>8-piece package</x:v>
-      </x:c>
-      <x:c r="M6" s="32" t="n">
-        <x:v>8</x:v>
+      <x:c r="H6" s="47"/>
+      <x:c r="I6" s="47"/>
+      <x:c r="J6" s="48"/>
+      <x:c r="K6" s="49" t="str">
+        <x:f>IF(COUNTA(H6:J6)=0,"",C6*H6+D6*I6+E6*J6)</x:f>
+      </x:c>
+      <x:c r="L6" s="50" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="M6" s="56" t="str">
+        <x:v>Enter the unit prices for 8", 10" and 12" in columns H–J.</x:v>
       </x:c>
       <x:c r="N6" s="32" t="str">
         <x:v>4 × 8", 2 × 10", 2 × 12"</x:v>
       </x:c>
       <x:c r="O6" s="32" t="str">
+        <x:v>8-piece package</x:v>
+      </x:c>
+      <x:c r="P6" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="Q6" t="str">
+        <x:v>4 × 8", 2 × 10", 2 × 12"</x:v>
+      </x:c>
+      <x:c r="R6" t="str">
         <x:v>Standard</x:v>
       </x:c>
     </x:row>
@@ -668,26 +736,31 @@
       <x:c r="G7" s="15" t="str">
         <x:v>Silver Rounded Border</x:v>
       </x:c>
-      <x:c r="H7" s="39"/>
-      <x:c r="I7" s="40" t="str">
-        <x:f>IF(H7="","",F7*H7)</x:f>
-      </x:c>
-      <x:c r="J7" s="41" t="n">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="K7" s="46" t="str">
-        <x:v>Enter the per-frame unit price in column H.</x:v>
-      </x:c>
-      <x:c r="L7" s="32" t="str">
-        <x:v>10-piece package</x:v>
-      </x:c>
-      <x:c r="M7" s="32" t="n">
-        <x:v>10</x:v>
+      <x:c r="H7" s="47"/>
+      <x:c r="I7" s="47"/>
+      <x:c r="J7" s="48"/>
+      <x:c r="K7" s="49" t="str">
+        <x:f>IF(COUNTA(H7:J7)=0,"",C7*H7+D7*I7+E7*J7)</x:f>
+      </x:c>
+      <x:c r="L7" s="50" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="M7" s="56" t="str">
+        <x:v>Enter the unit prices for 8", 10" and 12" in columns H–J.</x:v>
       </x:c>
       <x:c r="N7" s="32" t="str">
         <x:v>6 × 8", 2 × 10", 2 × 12"</x:v>
       </x:c>
       <x:c r="O7" s="35" t="str">
+        <x:v>10-piece package</x:v>
+      </x:c>
+      <x:c r="P7" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="Q7" t="str">
+        <x:v>6 × 8", 2 × 10", 2 × 12"</x:v>
+      </x:c>
+      <x:c r="R7" t="str">
         <x:v>Most Popular</x:v>
       </x:c>
     </x:row>
@@ -713,16 +786,22 @@
       <x:c r="G8" s="15" t="str">
         <x:v>Black Rounded Border</x:v>
       </x:c>
-      <x:c r="H8" s="39"/>
-      <x:c r="I8" s="40" t="str">
-        <x:f>IF(H8="","",F8*H8)</x:f>
-      </x:c>
-      <x:c r="J8" s="41" t="n">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="K8" s="46" t="str">
-        <x:v>Enter the per-frame unit price in column H.</x:v>
-      </x:c>
+      <x:c r="H8" s="47"/>
+      <x:c r="I8" s="47"/>
+      <x:c r="J8" s="48"/>
+      <x:c r="K8" s="49" t="str">
+        <x:f>IF(COUNTA(H8:J8)=0,"",C8*H8+D8*I8+E8*J8)</x:f>
+      </x:c>
+      <x:c r="L8" s="51" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="M8" s="46" t="str">
+        <x:v>Enter the unit prices for 8", 10" and 12" in columns H–J.</x:v>
+      </x:c>
+      <x:c r="O8"/>
+      <x:c r="P8"/>
+      <x:c r="Q8"/>
+      <x:c r="R8"/>
     </x:row>
     <x:row r="9" ht="24" customHeight="1">
       <x:c r="A9" s="15" t="str">
@@ -746,22 +825,25 @@
       <x:c r="G9" s="15" t="str">
         <x:v>Gold Square Corner</x:v>
       </x:c>
-      <x:c r="H9" s="39"/>
-      <x:c r="I9" s="40" t="str">
-        <x:f>IF(H9="","",F9*H9)</x:f>
-      </x:c>
-      <x:c r="J9" s="41" t="n">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="K9" s="46" t="str">
-        <x:v>Enter the per-frame unit price in column H.</x:v>
-      </x:c>
-      <x:c r="L9" s="37" t="str">
+      <x:c r="H9" s="47"/>
+      <x:c r="I9" s="47"/>
+      <x:c r="J9" s="48"/>
+      <x:c r="K9" s="49" t="str">
+        <x:f>IF(COUNTA(H9:J9)=0,"",C9*H9+D9*I9+E9*J9)</x:f>
+      </x:c>
+      <x:c r="L9" s="52" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="M9" s="57" t="str">
+        <x:v>Enter the unit prices for 8", 10" and 12" in columns H–J.</x:v>
+      </x:c>
+      <x:c r="N9" s="37"/>
+      <x:c r="O9" s="37" t="str">
         <x:v>Material names match the folders in public/frame-products.</x:v>
       </x:c>
-      <x:c r="M9" s="37"/>
-      <x:c r="N9" s="37"/>
-      <x:c r="O9" s="37"/>
+      <x:c r="P9"/>
+      <x:c r="Q9"/>
+      <x:c r="R9"/>
     </x:row>
     <x:row r="10" ht="24" customHeight="1">
       <x:c r="A10" s="15" t="str">
@@ -785,15 +867,17 @@
       <x:c r="G10" s="15" t="str">
         <x:v>Solid Wood - Warm Walnut</x:v>
       </x:c>
-      <x:c r="H10" s="39"/>
-      <x:c r="I10" s="40" t="str">
-        <x:f>IF(H10="","",F10*H10)</x:f>
-      </x:c>
-      <x:c r="J10" s="41" t="n">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="K10" s="46" t="str">
-        <x:v>Enter the per-frame unit price in column H.</x:v>
+      <x:c r="H10" s="47"/>
+      <x:c r="I10" s="47"/>
+      <x:c r="J10" s="48"/>
+      <x:c r="K10" s="49" t="str">
+        <x:f>IF(COUNTA(H10:J10)=0,"",C10*H10+D10*I10+E10*J10)</x:f>
+      </x:c>
+      <x:c r="L10" s="51" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="M10" s="46" t="str">
+        <x:v>Enter the unit prices for 8", 10" and 12" in columns H–J.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="24" customHeight="1">
@@ -818,15 +902,17 @@
       <x:c r="G11" s="15" t="str">
         <x:v>Fresh Light Wheat</x:v>
       </x:c>
-      <x:c r="H11" s="39"/>
-      <x:c r="I11" s="40" t="str">
-        <x:f>IF(H11="","",F11*H11)</x:f>
-      </x:c>
-      <x:c r="J11" s="41" t="n">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="K11" s="46" t="str">
-        <x:v>Enter the per-frame unit price in column H.</x:v>
+      <x:c r="H11" s="47"/>
+      <x:c r="I11" s="47"/>
+      <x:c r="J11" s="48"/>
+      <x:c r="K11" s="49" t="str">
+        <x:f>IF(COUNTA(H11:J11)=0,"",C11*H11+D11*I11+E11*J11)</x:f>
+      </x:c>
+      <x:c r="L11" s="51" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="M11" s="46" t="str">
+        <x:v>Enter the unit prices for 8", 10" and 12" in columns H–J.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="24" customHeight="1">
@@ -851,15 +937,17 @@
       <x:c r="G12" s="15" t="str">
         <x:v>Roasted Tea</x:v>
       </x:c>
-      <x:c r="H12" s="39"/>
-      <x:c r="I12" s="40" t="str">
-        <x:f>IF(H12="","",F12*H12)</x:f>
-      </x:c>
-      <x:c r="J12" s="41" t="n">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="K12" s="46" t="str">
-        <x:v>Enter the per-frame unit price in column H.</x:v>
+      <x:c r="H12" s="47"/>
+      <x:c r="I12" s="47"/>
+      <x:c r="J12" s="48"/>
+      <x:c r="K12" s="49" t="str">
+        <x:f>IF(COUNTA(H12:J12)=0,"",C12*H12+D12*I12+E12*J12)</x:f>
+      </x:c>
+      <x:c r="L12" s="51" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="M12" s="46" t="str">
+        <x:v>Enter the unit prices for 8", 10" and 12" in columns H–J.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="24" customHeight="1">
@@ -884,15 +972,17 @@
       <x:c r="G13" s="15" t="str">
         <x:v>Black Walnut</x:v>
       </x:c>
-      <x:c r="H13" s="39"/>
-      <x:c r="I13" s="40" t="str">
-        <x:f>IF(H13="","",F13*H13)</x:f>
-      </x:c>
-      <x:c r="J13" s="41" t="n">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="K13" s="46" t="str">
-        <x:v>Enter the per-frame unit price in column H.</x:v>
+      <x:c r="H13" s="47"/>
+      <x:c r="I13" s="47"/>
+      <x:c r="J13" s="48"/>
+      <x:c r="K13" s="49" t="str">
+        <x:f>IF(COUNTA(H13:J13)=0,"",C13*H13+D13*I13+E13*J13)</x:f>
+      </x:c>
+      <x:c r="L13" s="51" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="M13" s="46" t="str">
+        <x:v>Enter the unit prices for 8", 10" and 12" in columns H–J.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="24" customHeight="1">
@@ -917,15 +1007,17 @@
       <x:c r="G14" s="15" t="str">
         <x:v>Frameless Rounded Corner</x:v>
       </x:c>
-      <x:c r="H14" s="39"/>
-      <x:c r="I14" s="40" t="str">
-        <x:f>IF(H14="","",F14*H14)</x:f>
-      </x:c>
-      <x:c r="J14" s="41" t="n">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="K14" s="46" t="str">
-        <x:v>Enter the per-frame unit price in column H.</x:v>
+      <x:c r="H14" s="47"/>
+      <x:c r="I14" s="47"/>
+      <x:c r="J14" s="48"/>
+      <x:c r="K14" s="49" t="str">
+        <x:f>IF(COUNTA(H14:J14)=0,"",C14*H14+D14*I14+E14*J14)</x:f>
+      </x:c>
+      <x:c r="L14" s="51" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="M14" s="46" t="str">
+        <x:v>Enter the unit prices for 8", 10" and 12" in columns H–J.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="24" customHeight="1">
@@ -950,15 +1042,17 @@
       <x:c r="G15" s="15" t="str">
         <x:v>White Rounded Border</x:v>
       </x:c>
-      <x:c r="H15" s="39"/>
-      <x:c r="I15" s="40" t="str">
-        <x:f>IF(H15="","",F15*H15)</x:f>
-      </x:c>
-      <x:c r="J15" s="41" t="n">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="K15" s="46" t="str">
-        <x:v>Enter the per-frame unit price in column H.</x:v>
+      <x:c r="H15" s="47"/>
+      <x:c r="I15" s="47"/>
+      <x:c r="J15" s="48"/>
+      <x:c r="K15" s="49" t="str">
+        <x:f>IF(COUNTA(H15:J15)=0,"",C15*H15+D15*I15+E15*J15)</x:f>
+      </x:c>
+      <x:c r="L15" s="51" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="M15" s="46" t="str">
+        <x:v>Enter the unit prices for 8", 10" and 12" in columns H–J.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="24" customHeight="1">
@@ -983,15 +1077,17 @@
       <x:c r="G16" s="15" t="str">
         <x:v>Silver Rounded Border</x:v>
       </x:c>
-      <x:c r="H16" s="39"/>
-      <x:c r="I16" s="40" t="str">
-        <x:f>IF(H16="","",F16*H16)</x:f>
-      </x:c>
-      <x:c r="J16" s="41" t="n">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="K16" s="46" t="str">
-        <x:v>Enter the per-frame unit price in column H.</x:v>
+      <x:c r="H16" s="47"/>
+      <x:c r="I16" s="47"/>
+      <x:c r="J16" s="48"/>
+      <x:c r="K16" s="49" t="str">
+        <x:f>IF(COUNTA(H16:J16)=0,"",C16*H16+D16*I16+E16*J16)</x:f>
+      </x:c>
+      <x:c r="L16" s="51" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="M16" s="46" t="str">
+        <x:v>Enter the unit prices for 8", 10" and 12" in columns H–J.</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="24" customHeight="1">
@@ -1016,15 +1112,17 @@
       <x:c r="G17" s="15" t="str">
         <x:v>Black Rounded Border</x:v>
       </x:c>
-      <x:c r="H17" s="39"/>
-      <x:c r="I17" s="40" t="str">
-        <x:f>IF(H17="","",F17*H17)</x:f>
-      </x:c>
-      <x:c r="J17" s="41" t="n">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="K17" s="46" t="str">
-        <x:v>Enter the per-frame unit price in column H.</x:v>
+      <x:c r="H17" s="47"/>
+      <x:c r="I17" s="47"/>
+      <x:c r="J17" s="48"/>
+      <x:c r="K17" s="49" t="str">
+        <x:f>IF(COUNTA(H17:J17)=0,"",C17*H17+D17*I17+E17*J17)</x:f>
+      </x:c>
+      <x:c r="L17" s="51" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="M17" s="46" t="str">
+        <x:v>Enter the unit prices for 8", 10" and 12" in columns H–J.</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="24" customHeight="1">
@@ -1049,15 +1147,17 @@
       <x:c r="G18" s="15" t="str">
         <x:v>Gold Square Corner</x:v>
       </x:c>
-      <x:c r="H18" s="39"/>
-      <x:c r="I18" s="40" t="str">
-        <x:f>IF(H18="","",F18*H18)</x:f>
-      </x:c>
-      <x:c r="J18" s="41" t="n">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="K18" s="46" t="str">
-        <x:v>Enter the per-frame unit price in column H.</x:v>
+      <x:c r="H18" s="47"/>
+      <x:c r="I18" s="47"/>
+      <x:c r="J18" s="48"/>
+      <x:c r="K18" s="49" t="str">
+        <x:f>IF(COUNTA(H18:J18)=0,"",C18*H18+D18*I18+E18*J18)</x:f>
+      </x:c>
+      <x:c r="L18" s="51" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="M18" s="46" t="str">
+        <x:v>Enter the unit prices for 8", 10" and 12" in columns H–J.</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="24" customHeight="1">
@@ -1082,15 +1182,17 @@
       <x:c r="G19" s="15" t="str">
         <x:v>Solid Wood - Warm Walnut</x:v>
       </x:c>
-      <x:c r="H19" s="39"/>
-      <x:c r="I19" s="40" t="str">
-        <x:f>IF(H19="","",F19*H19)</x:f>
-      </x:c>
-      <x:c r="J19" s="41" t="n">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="K19" s="46" t="str">
-        <x:v>Enter the per-frame unit price in column H.</x:v>
+      <x:c r="H19" s="47"/>
+      <x:c r="I19" s="47"/>
+      <x:c r="J19" s="48"/>
+      <x:c r="K19" s="49" t="str">
+        <x:f>IF(COUNTA(H19:J19)=0,"",C19*H19+D19*I19+E19*J19)</x:f>
+      </x:c>
+      <x:c r="L19" s="51" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="M19" s="46" t="str">
+        <x:v>Enter the unit prices for 8", 10" and 12" in columns H–J.</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="24" customHeight="1">
@@ -1115,15 +1217,17 @@
       <x:c r="G20" s="15" t="str">
         <x:v>Fresh Light Wheat</x:v>
       </x:c>
-      <x:c r="H20" s="39"/>
-      <x:c r="I20" s="40" t="str">
-        <x:f>IF(H20="","",F20*H20)</x:f>
-      </x:c>
-      <x:c r="J20" s="41" t="n">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="K20" s="46" t="str">
-        <x:v>Enter the per-frame unit price in column H.</x:v>
+      <x:c r="H20" s="47"/>
+      <x:c r="I20" s="47"/>
+      <x:c r="J20" s="48"/>
+      <x:c r="K20" s="49" t="str">
+        <x:f>IF(COUNTA(H20:J20)=0,"",C20*H20+D20*I20+E20*J20)</x:f>
+      </x:c>
+      <x:c r="L20" s="51" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="M20" s="46" t="str">
+        <x:v>Enter the unit prices for 8", 10" and 12" in columns H–J.</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="24" customHeight="1">
@@ -1148,15 +1252,17 @@
       <x:c r="G21" s="15" t="str">
         <x:v>Roasted Tea</x:v>
       </x:c>
-      <x:c r="H21" s="39"/>
-      <x:c r="I21" s="40" t="str">
-        <x:f>IF(H21="","",F21*H21)</x:f>
-      </x:c>
-      <x:c r="J21" s="41" t="n">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="K21" s="46" t="str">
-        <x:v>Enter the per-frame unit price in column H.</x:v>
+      <x:c r="H21" s="47"/>
+      <x:c r="I21" s="47"/>
+      <x:c r="J21" s="48"/>
+      <x:c r="K21" s="49" t="str">
+        <x:f>IF(COUNTA(H21:J21)=0,"",C21*H21+D21*I21+E21*J21)</x:f>
+      </x:c>
+      <x:c r="L21" s="51" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="M21" s="46" t="str">
+        <x:v>Enter the unit prices for 8", 10" and 12" in columns H–J.</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="24" customHeight="1">
@@ -1181,15 +1287,17 @@
       <x:c r="G22" s="15" t="str">
         <x:v>Black Walnut</x:v>
       </x:c>
-      <x:c r="H22" s="39"/>
-      <x:c r="I22" s="40" t="str">
-        <x:f>IF(H22="","",F22*H22)</x:f>
-      </x:c>
-      <x:c r="J22" s="41" t="n">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="K22" s="46" t="str">
-        <x:v>Enter the per-frame unit price in column H.</x:v>
+      <x:c r="H22" s="47"/>
+      <x:c r="I22" s="47"/>
+      <x:c r="J22" s="48"/>
+      <x:c r="K22" s="49" t="str">
+        <x:f>IF(COUNTA(H22:J22)=0,"",C22*H22+D22*I22+E22*J22)</x:f>
+      </x:c>
+      <x:c r="L22" s="51" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="M22" s="46" t="str">
+        <x:v>Enter the unit prices for 8", 10" and 12" in columns H–J.</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="24" customHeight="1">
@@ -1214,15 +1322,17 @@
       <x:c r="G23" s="15" t="str">
         <x:v>Frameless Rounded Corner</x:v>
       </x:c>
-      <x:c r="H23" s="39"/>
-      <x:c r="I23" s="40" t="str">
-        <x:f>IF(H23="","",F23*H23)</x:f>
-      </x:c>
-      <x:c r="J23" s="41" t="n">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="K23" s="46" t="str">
-        <x:v>Enter the per-frame unit price in column H.</x:v>
+      <x:c r="H23" s="47"/>
+      <x:c r="I23" s="47"/>
+      <x:c r="J23" s="48"/>
+      <x:c r="K23" s="49" t="str">
+        <x:f>IF(COUNTA(H23:J23)=0,"",C23*H23+D23*I23+E23*J23)</x:f>
+      </x:c>
+      <x:c r="L23" s="51" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="M23" s="46" t="str">
+        <x:v>Enter the unit prices for 8", 10" and 12" in columns H–J.</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="24" customHeight="1">
@@ -1247,15 +1357,17 @@
       <x:c r="G24" s="15" t="str">
         <x:v>White Rounded Border</x:v>
       </x:c>
-      <x:c r="H24" s="39"/>
-      <x:c r="I24" s="40" t="str">
-        <x:f>IF(H24="","",F24*H24)</x:f>
-      </x:c>
-      <x:c r="J24" s="41" t="n">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="K24" s="46" t="str">
-        <x:v>Enter the per-frame unit price in column H.</x:v>
+      <x:c r="H24" s="47"/>
+      <x:c r="I24" s="47"/>
+      <x:c r="J24" s="48"/>
+      <x:c r="K24" s="49" t="str">
+        <x:f>IF(COUNTA(H24:J24)=0,"",C24*H24+D24*I24+E24*J24)</x:f>
+      </x:c>
+      <x:c r="L24" s="51" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="M24" s="46" t="str">
+        <x:v>Enter the unit prices for 8", 10" and 12" in columns H–J.</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="24" customHeight="1">
@@ -1280,15 +1392,17 @@
       <x:c r="G25" s="15" t="str">
         <x:v>Silver Rounded Border</x:v>
       </x:c>
-      <x:c r="H25" s="39"/>
-      <x:c r="I25" s="40" t="str">
-        <x:f>IF(H25="","",F25*H25)</x:f>
-      </x:c>
-      <x:c r="J25" s="41" t="n">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="K25" s="46" t="str">
-        <x:v>Enter the per-frame unit price in column H.</x:v>
+      <x:c r="H25" s="47"/>
+      <x:c r="I25" s="47"/>
+      <x:c r="J25" s="48"/>
+      <x:c r="K25" s="49" t="str">
+        <x:f>IF(COUNTA(H25:J25)=0,"",C25*H25+D25*I25+E25*J25)</x:f>
+      </x:c>
+      <x:c r="L25" s="51" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="M25" s="46" t="str">
+        <x:v>Enter the unit prices for 8", 10" and 12" in columns H–J.</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="24" customHeight="1">
@@ -1313,15 +1427,17 @@
       <x:c r="G26" s="15" t="str">
         <x:v>Black Rounded Border</x:v>
       </x:c>
-      <x:c r="H26" s="39"/>
-      <x:c r="I26" s="40" t="str">
-        <x:f>IF(H26="","",F26*H26)</x:f>
-      </x:c>
-      <x:c r="J26" s="41" t="n">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="K26" s="46" t="str">
-        <x:v>Enter the per-frame unit price in column H.</x:v>
+      <x:c r="H26" s="47"/>
+      <x:c r="I26" s="47"/>
+      <x:c r="J26" s="48"/>
+      <x:c r="K26" s="49" t="str">
+        <x:f>IF(COUNTA(H26:J26)=0,"",C26*H26+D26*I26+E26*J26)</x:f>
+      </x:c>
+      <x:c r="L26" s="51" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="M26" s="46" t="str">
+        <x:v>Enter the unit prices for 8", 10" and 12" in columns H–J.</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="24" customHeight="1">
@@ -1346,15 +1462,17 @@
       <x:c r="G27" s="15" t="str">
         <x:v>Gold Square Corner</x:v>
       </x:c>
-      <x:c r="H27" s="39"/>
-      <x:c r="I27" s="40" t="str">
-        <x:f>IF(H27="","",F27*H27)</x:f>
-      </x:c>
-      <x:c r="J27" s="41" t="n">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="K27" s="46" t="str">
-        <x:v>Enter the per-frame unit price in column H.</x:v>
+      <x:c r="H27" s="47"/>
+      <x:c r="I27" s="47"/>
+      <x:c r="J27" s="48"/>
+      <x:c r="K27" s="49" t="str">
+        <x:f>IF(COUNTA(H27:J27)=0,"",C27*H27+D27*I27+E27*J27)</x:f>
+      </x:c>
+      <x:c r="L27" s="51" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="M27" s="46" t="str">
+        <x:v>Enter the unit prices for 8", 10" and 12" in columns H–J.</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="24" customHeight="1">
@@ -1379,15 +1497,17 @@
       <x:c r="G28" s="15" t="str">
         <x:v>Solid Wood - Warm Walnut</x:v>
       </x:c>
-      <x:c r="H28" s="39"/>
-      <x:c r="I28" s="40" t="str">
-        <x:f>IF(H28="","",F28*H28)</x:f>
-      </x:c>
-      <x:c r="J28" s="41" t="n">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="K28" s="46" t="str">
-        <x:v>Enter the per-frame unit price in column H.</x:v>
+      <x:c r="H28" s="47"/>
+      <x:c r="I28" s="47"/>
+      <x:c r="J28" s="48"/>
+      <x:c r="K28" s="49" t="str">
+        <x:f>IF(COUNTA(H28:J28)=0,"",C28*H28+D28*I28+E28*J28)</x:f>
+      </x:c>
+      <x:c r="L28" s="51" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="M28" s="46" t="str">
+        <x:v>Enter the unit prices for 8", 10" and 12" in columns H–J.</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="24" customHeight="1">
@@ -1412,15 +1532,17 @@
       <x:c r="G29" s="15" t="str">
         <x:v>Fresh Light Wheat</x:v>
       </x:c>
-      <x:c r="H29" s="39"/>
-      <x:c r="I29" s="40" t="str">
-        <x:f>IF(H29="","",F29*H29)</x:f>
-      </x:c>
-      <x:c r="J29" s="41" t="n">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="K29" s="46" t="str">
-        <x:v>Enter the per-frame unit price in column H.</x:v>
+      <x:c r="H29" s="47"/>
+      <x:c r="I29" s="47"/>
+      <x:c r="J29" s="48"/>
+      <x:c r="K29" s="49" t="str">
+        <x:f>IF(COUNTA(H29:J29)=0,"",C29*H29+D29*I29+E29*J29)</x:f>
+      </x:c>
+      <x:c r="L29" s="51" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="M29" s="46" t="str">
+        <x:v>Enter the unit prices for 8", 10" and 12" in columns H–J.</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="24" customHeight="1">
@@ -1445,15 +1567,17 @@
       <x:c r="G30" s="15" t="str">
         <x:v>Roasted Tea</x:v>
       </x:c>
-      <x:c r="H30" s="39"/>
-      <x:c r="I30" s="40" t="str">
-        <x:f>IF(H30="","",F30*H30)</x:f>
-      </x:c>
-      <x:c r="J30" s="41" t="n">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="K30" s="46" t="str">
-        <x:v>Enter the per-frame unit price in column H.</x:v>
+      <x:c r="H30" s="47"/>
+      <x:c r="I30" s="47"/>
+      <x:c r="J30" s="48"/>
+      <x:c r="K30" s="49" t="str">
+        <x:f>IF(COUNTA(H30:J30)=0,"",C30*H30+D30*I30+E30*J30)</x:f>
+      </x:c>
+      <x:c r="L30" s="51" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="M30" s="46" t="str">
+        <x:v>Enter the unit prices for 8", 10" and 12" in columns H–J.</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="24" customHeight="1">
@@ -1478,15 +1602,17 @@
       <x:c r="G31" s="15" t="str">
         <x:v>Black Walnut</x:v>
       </x:c>
-      <x:c r="H31" s="39"/>
-      <x:c r="I31" s="40" t="str">
-        <x:f>IF(H31="","",F31*H31)</x:f>
-      </x:c>
-      <x:c r="J31" s="41" t="n">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="K31" s="46" t="str">
-        <x:v>Enter the per-frame unit price in column H.</x:v>
+      <x:c r="H31" s="47"/>
+      <x:c r="I31" s="47"/>
+      <x:c r="J31" s="48"/>
+      <x:c r="K31" s="49" t="str">
+        <x:f>IF(COUNTA(H31:J31)=0,"",C31*H31+D31*I31+E31*J31)</x:f>
+      </x:c>
+      <x:c r="L31" s="51" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="M31" s="46" t="str">
+        <x:v>Enter the unit prices for 8", 10" and 12" in columns H–J.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Fix A4 pricing formulas across all rows
</commit_message>
<xml_diff>
--- a/apps/moment-booth-fe/data/frame-package-pricing.xlsx
+++ b/apps/moment-booth-fe/data/frame-package-pricing.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Frame Pricing" sheetId="1" r:id="R511bf13e3e1e49e3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Frame Pricing" sheetId="1" r:id="Rc0b8f6eec71642d9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1507,7 +1507,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="M6" s="13" t="n">
-        <x:f>IF(COUNTA(I6:K6)=0,"",C6*I6+D6*J6+E6*K6)</x:f>
+        <x:f>IF(COUNTA(I6:L6)=0,"",C6*I6+D6*J6+E6*K6+F6*L6)</x:f>
         <x:v>94</x:v>
       </x:c>
       <x:c r="N6" s="14" t="n">
@@ -1571,7 +1571,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="M7" s="13" t="n">
-        <x:f>IF(COUNTA(I7:K7)=0,"",C7*I7+D7*J7+E7*K7)</x:f>
+        <x:f>IF(COUNTA(I7:L7)=0,"",C7*I7+D7*J7+E7*K7+F7*L7)</x:f>
         <x:v>94</x:v>
       </x:c>
       <x:c r="N7" s="14">
@@ -1635,7 +1635,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="M8" s="13" t="n">
-        <x:f>IF(COUNTA(I8:K8)=0,"",C8*I8+D8*J8+E8*K8)</x:f>
+        <x:f>IF(COUNTA(I8:L8)=0,"",C8*I8+D8*J8+E8*K8+F8*L8)</x:f>
         <x:v>94</x:v>
       </x:c>
       <x:c r="N8" s="14">
@@ -1684,7 +1684,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="M9" s="13" t="n">
-        <x:f>IF(COUNTA(I9:K9)=0,"",C9*I9+D9*J9+E9*K9)</x:f>
+        <x:f>IF(COUNTA(I9:L9)=0,"",C9*I9+D9*J9+E9*K9+F9*L9)</x:f>
         <x:v>172</x:v>
       </x:c>
       <x:c r="N9" s="14">
@@ -1737,8 +1737,8 @@
         <x:v>34</x:v>
       </x:c>
       <x:c r="M10" s="13" t="n">
-        <x:f>IF(COUNTA(I10:K10)=0,"",C10*I10+D10*J10+E10*K10)</x:f>
-        <x:v>92</x:v>
+        <x:f>IF(COUNTA(I10:L10)=0,"",C10*I10+D10*J10+E10*K10+F10*L10)</x:f>
+        <x:v>160</x:v>
       </x:c>
       <x:c r="N10" s="14">
         <x:f t="shared" si="1"/>
@@ -1786,8 +1786,8 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="M11" s="13" t="n">
-        <x:f>IF(COUNTA(I11:K11)=0,"",C11*I11+D11*J11+E11*K11)</x:f>
-        <x:v>88</x:v>
+        <x:f>IF(COUNTA(I11:L11)=0,"",C11*I11+D11*J11+E11*K11+F11*L11)</x:f>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="N11" s="14">
         <x:f t="shared" si="1"/>
@@ -1835,8 +1835,8 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="M12" s="13" t="n">
-        <x:f>IF(COUNTA(I12:K12)=0,"",C12*I12+D12*J12+E12*K12)</x:f>
-        <x:v>88</x:v>
+        <x:f>IF(COUNTA(I12:L12)=0,"",C12*I12+D12*J12+E12*K12+F12*L12)</x:f>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="N12" s="14">
         <x:f t="shared" si="1"/>
@@ -1884,8 +1884,8 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="M13" s="13" t="n">
-        <x:f>IF(COUNTA(I13:K13)=0,"",C13*I13+D13*J13+E13*K13)</x:f>
-        <x:v>88</x:v>
+        <x:f>IF(COUNTA(I13:L13)=0,"",C13*I13+D13*J13+E13*K13+F13*L13)</x:f>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="N13" s="14">
         <x:f t="shared" si="1"/>
@@ -1933,7 +1933,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="M14" s="13" t="n">
-        <x:f>IF(COUNTA(I14:K14)=0,"",C14*I14+D14*J14+E14*K14)</x:f>
+        <x:f>IF(COUNTA(I14:L14)=0,"",C14*I14+D14*J14+E14*K14+F14*L14)</x:f>
         <x:v>128</x:v>
       </x:c>
       <x:c r="N14" s="14">
@@ -1982,7 +1982,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="M15" s="13" t="n">
-        <x:f>IF(COUNTA(I15:K15)=0,"",C15*I15+D15*J15+E15*K15)</x:f>
+        <x:f>IF(COUNTA(I15:L15)=0,"",C15*I15+D15*J15+E15*K15+F15*L15)</x:f>
         <x:v>120</x:v>
       </x:c>
       <x:c r="N15" s="14">
@@ -2031,7 +2031,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="M16" s="13" t="n">
-        <x:f>IF(COUNTA(I16:K16)=0,"",C16*I16+D16*J16+E16*K16)</x:f>
+        <x:f>IF(COUNTA(I16:L16)=0,"",C16*I16+D16*J16+E16*K16+F16*L16)</x:f>
         <x:v>120</x:v>
       </x:c>
       <x:c r="N16" s="14">
@@ -2080,7 +2080,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="M17" s="13" t="n">
-        <x:f>IF(COUNTA(I17:K17)=0,"",C17*I17+D17*J17+E17*K17)</x:f>
+        <x:f>IF(COUNTA(I17:L17)=0,"",C17*I17+D17*J17+E17*K17+F17*L17)</x:f>
         <x:v>120</x:v>
       </x:c>
       <x:c r="N17" s="14">
@@ -2129,7 +2129,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="M18" s="13" t="n">
-        <x:f>IF(COUNTA(I18:K18)=0,"",C18*I18+D18*J18+E18*K18)</x:f>
+        <x:f>IF(COUNTA(I18:L18)=0,"",C18*I18+D18*J18+E18*K18+F18*L18)</x:f>
         <x:v>220</x:v>
       </x:c>
       <x:c r="N18" s="14">
@@ -2178,8 +2178,8 @@
         <x:v>34</x:v>
       </x:c>
       <x:c r="M19" s="13" t="n">
-        <x:f>IF(COUNTA(I19:K19)=0,"",C19*I19+D19*J19+E19*K19)</x:f>
-        <x:v>132</x:v>
+        <x:f>IF(COUNTA(I19:L19)=0,"",C19*I19+D19*J19+E19*K19+F19*L19)</x:f>
+        <x:v>200</x:v>
       </x:c>
       <x:c r="N19" s="14">
         <x:f t="shared" si="1"/>
@@ -2227,8 +2227,8 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="M20" s="13" t="n">
-        <x:f>IF(COUNTA(I20:K20)=0,"",C20*I20+D20*J20+E20*K20)</x:f>
-        <x:v>124</x:v>
+        <x:f>IF(COUNTA(I20:L20)=0,"",C20*I20+D20*J20+E20*K20+F20*L20)</x:f>
+        <x:v>184</x:v>
       </x:c>
       <x:c r="N20" s="14">
         <x:f t="shared" si="1"/>
@@ -2276,8 +2276,8 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="M21" s="13" t="n">
-        <x:f>IF(COUNTA(I21:K21)=0,"",C21*I21+D21*J21+E21*K21)</x:f>
-        <x:v>124</x:v>
+        <x:f>IF(COUNTA(I21:L21)=0,"",C21*I21+D21*J21+E21*K21+F21*L21)</x:f>
+        <x:v>184</x:v>
       </x:c>
       <x:c r="N21" s="14">
         <x:f t="shared" si="1"/>
@@ -2325,8 +2325,8 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="M22" s="13" t="n">
-        <x:f>IF(COUNTA(I22:K22)=0,"",C22*I22+D22*J22+E22*K22)</x:f>
-        <x:v>124</x:v>
+        <x:f>IF(COUNTA(I22:L22)=0,"",C22*I22+D22*J22+E22*K22+F22*L22)</x:f>
+        <x:v>184</x:v>
       </x:c>
       <x:c r="N22" s="14">
         <x:f t="shared" si="1"/>
@@ -2374,7 +2374,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="M23" s="13" t="n">
-        <x:f>IF(COUNTA(I23:K23)=0,"",C23*I23+D23*J23+E23*K23)</x:f>
+        <x:f>IF(COUNTA(I23:L23)=0,"",C23*I23+D23*J23+E23*K23+F23*L23)</x:f>
         <x:v>154</x:v>
       </x:c>
       <x:c r="N23" s="14">
@@ -2423,7 +2423,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="M24" s="13" t="n">
-        <x:f>IF(COUNTA(I24:K24)=0,"",C24*I24+D24*J24+E24*K24)</x:f>
+        <x:f>IF(COUNTA(I24:L24)=0,"",C24*I24+D24*J24+E24*K24+F24*L24)</x:f>
         <x:v>146</x:v>
       </x:c>
       <x:c r="N24" s="14">
@@ -2472,7 +2472,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="M25" s="13" t="n">
-        <x:f>IF(COUNTA(I25:K25)=0,"",C25*I25+D25*J25+E25*K25)</x:f>
+        <x:f>IF(COUNTA(I25:L25)=0,"",C25*I25+D25*J25+E25*K25+F25*L25)</x:f>
         <x:v>146</x:v>
       </x:c>
       <x:c r="N25" s="14">
@@ -2521,7 +2521,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="M26" s="13" t="n">
-        <x:f>IF(COUNTA(I26:K26)=0,"",C26*I26+D26*J26+E26*K26)</x:f>
+        <x:f>IF(COUNTA(I26:L26)=0,"",C26*I26+D26*J26+E26*K26+F26*L26)</x:f>
         <x:v>146</x:v>
       </x:c>
       <x:c r="N26" s="14">
@@ -2570,7 +2570,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="M27" s="13" t="n">
-        <x:f>IF(COUNTA(I27:K27)=0,"",C27*I27+D27*J27+E27*K27)</x:f>
+        <x:f>IF(COUNTA(I27:L27)=0,"",C27*I27+D27*J27+E27*K27+F27*L27)</x:f>
         <x:v>268</x:v>
       </x:c>
       <x:c r="N27" s="14">
@@ -2619,8 +2619,8 @@
         <x:v>34</x:v>
       </x:c>
       <x:c r="M28" s="13" t="n">
-        <x:f>IF(COUNTA(I28:K28)=0,"",C28*I28+D28*J28+E28*K28)</x:f>
-        <x:v>172</x:v>
+        <x:f>IF(COUNTA(I28:L28)=0,"",C28*I28+D28*J28+E28*K28+F28*L28)</x:f>
+        <x:v>240</x:v>
       </x:c>
       <x:c r="N28" s="14">
         <x:f t="shared" si="1"/>
@@ -2668,8 +2668,8 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="M29" s="13" t="n">
-        <x:f>IF(COUNTA(I29:K29)=0,"",C29*I29+D29*J29+E29*K29)</x:f>
-        <x:v>160</x:v>
+        <x:f>IF(COUNTA(I29:L29)=0,"",C29*I29+D29*J29+E29*K29+F29*L29)</x:f>
+        <x:v>220</x:v>
       </x:c>
       <x:c r="N29" s="14">
         <x:f t="shared" si="1"/>
@@ -2717,8 +2717,8 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="M30" s="13" t="n">
-        <x:f>IF(COUNTA(I30:K30)=0,"",C30*I30+D30*J30+E30*K30)</x:f>
-        <x:v>160</x:v>
+        <x:f>IF(COUNTA(I30:L30)=0,"",C30*I30+D30*J30+E30*K30+F30*L30)</x:f>
+        <x:v>220</x:v>
       </x:c>
       <x:c r="N30" s="14">
         <x:f t="shared" si="1"/>
@@ -2766,8 +2766,8 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="M31" s="13" t="n">
-        <x:f>IF(COUNTA(I31:K31)=0,"",C31*I31+D31*J31+E31*K31)</x:f>
-        <x:v>160</x:v>
+        <x:f>IF(COUNTA(I31:L31)=0,"",C31*I31+D31*J31+E31*K31+F31*L31)</x:f>
+        <x:v>220</x:v>
       </x:c>
       <x:c r="N31" s="14">
         <x:f t="shared" si="1"/>

</xml_diff>

<commit_message>
Format synced prices to two decimals
</commit_message>
<xml_diff>
--- a/apps/moment-booth-fe/data/frame-package-pricing.xlsx
+++ b/apps/moment-booth-fe/data/frame-package-pricing.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Frame Pricing" sheetId="1" r:id="Rc0b8f6eec71642d9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Frame Pricing" sheetId="1" r:id="Rd3442a270afe42b4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1443,7 +1443,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="M5" s="13" t="n">
-        <x:f t="shared" ref="M5" si="0">IF(COUNTA(I5:L5)=0,"",C5*I5+D5*J5+E5*K5+F5*L5)</x:f>
+        <x:f t="shared" ref="M5" si="0">IF(COUNTA(I5:L5)=0,"",ROUND(C5*I5+D5*J5+E5*K5+F5*L5,2))</x:f>
         <x:v>102</x:v>
       </x:c>
       <x:c r="N5" s="14" t="n">
@@ -1507,7 +1507,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="M6" s="13" t="n">
-        <x:f>IF(COUNTA(I6:L6)=0,"",C6*I6+D6*J6+E6*K6+F6*L6)</x:f>
+        <x:f>IF(COUNTA(I6:L6)=0,"",ROUND(C6*I6+D6*J6+E6*K6+F6*L6,2))</x:f>
         <x:v>94</x:v>
       </x:c>
       <x:c r="N6" s="14" t="n">
@@ -1571,7 +1571,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="M7" s="13" t="n">
-        <x:f>IF(COUNTA(I7:L7)=0,"",C7*I7+D7*J7+E7*K7+F7*L7)</x:f>
+        <x:f>IF(COUNTA(I7:L7)=0,"",ROUND(C7*I7+D7*J7+E7*K7+F7*L7,2))</x:f>
         <x:v>94</x:v>
       </x:c>
       <x:c r="N7" s="14">
@@ -1635,7 +1635,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="M8" s="13" t="n">
-        <x:f>IF(COUNTA(I8:L8)=0,"",C8*I8+D8*J8+E8*K8+F8*L8)</x:f>
+        <x:f>IF(COUNTA(I8:L8)=0,"",ROUND(C8*I8+D8*J8+E8*K8+F8*L8,2))</x:f>
         <x:v>94</x:v>
       </x:c>
       <x:c r="N8" s="14">
@@ -1684,7 +1684,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="M9" s="13" t="n">
-        <x:f>IF(COUNTA(I9:L9)=0,"",C9*I9+D9*J9+E9*K9+F9*L9)</x:f>
+        <x:f>IF(COUNTA(I9:L9)=0,"",ROUND(C9*I9+D9*J9+E9*K9+F9*L9,2))</x:f>
         <x:v>172</x:v>
       </x:c>
       <x:c r="N9" s="14">
@@ -1737,7 +1737,7 @@
         <x:v>34</x:v>
       </x:c>
       <x:c r="M10" s="13" t="n">
-        <x:f>IF(COUNTA(I10:L10)=0,"",C10*I10+D10*J10+E10*K10+F10*L10)</x:f>
+        <x:f>IF(COUNTA(I10:L10)=0,"",ROUND(C10*I10+D10*J10+E10*K10+F10*L10,2))</x:f>
         <x:v>160</x:v>
       </x:c>
       <x:c r="N10" s="14">
@@ -1786,7 +1786,7 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="M11" s="13" t="n">
-        <x:f>IF(COUNTA(I11:L11)=0,"",C11*I11+D11*J11+E11*K11+F11*L11)</x:f>
+        <x:f>IF(COUNTA(I11:L11)=0,"",ROUND(C11*I11+D11*J11+E11*K11+F11*L11,2))</x:f>
         <x:v>148</x:v>
       </x:c>
       <x:c r="N11" s="14">
@@ -1835,7 +1835,7 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="M12" s="13" t="n">
-        <x:f>IF(COUNTA(I12:L12)=0,"",C12*I12+D12*J12+E12*K12+F12*L12)</x:f>
+        <x:f>IF(COUNTA(I12:L12)=0,"",ROUND(C12*I12+D12*J12+E12*K12+F12*L12,2))</x:f>
         <x:v>148</x:v>
       </x:c>
       <x:c r="N12" s="14">
@@ -1884,7 +1884,7 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="M13" s="13" t="n">
-        <x:f>IF(COUNTA(I13:L13)=0,"",C13*I13+D13*J13+E13*K13+F13*L13)</x:f>
+        <x:f>IF(COUNTA(I13:L13)=0,"",ROUND(C13*I13+D13*J13+E13*K13+F13*L13,2))</x:f>
         <x:v>148</x:v>
       </x:c>
       <x:c r="N13" s="14">
@@ -1933,7 +1933,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="M14" s="13" t="n">
-        <x:f>IF(COUNTA(I14:L14)=0,"",C14*I14+D14*J14+E14*K14+F14*L14)</x:f>
+        <x:f>IF(COUNTA(I14:L14)=0,"",ROUND(C14*I14+D14*J14+E14*K14+F14*L14,2))</x:f>
         <x:v>128</x:v>
       </x:c>
       <x:c r="N14" s="14">
@@ -1982,7 +1982,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="M15" s="13" t="n">
-        <x:f>IF(COUNTA(I15:L15)=0,"",C15*I15+D15*J15+E15*K15+F15*L15)</x:f>
+        <x:f>IF(COUNTA(I15:L15)=0,"",ROUND(C15*I15+D15*J15+E15*K15+F15*L15,2))</x:f>
         <x:v>120</x:v>
       </x:c>
       <x:c r="N15" s="14">
@@ -2031,7 +2031,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="M16" s="13" t="n">
-        <x:f>IF(COUNTA(I16:L16)=0,"",C16*I16+D16*J16+E16*K16+F16*L16)</x:f>
+        <x:f>IF(COUNTA(I16:L16)=0,"",ROUND(C16*I16+D16*J16+E16*K16+F16*L16,2))</x:f>
         <x:v>120</x:v>
       </x:c>
       <x:c r="N16" s="14">
@@ -2080,7 +2080,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="M17" s="13" t="n">
-        <x:f>IF(COUNTA(I17:L17)=0,"",C17*I17+D17*J17+E17*K17+F17*L17)</x:f>
+        <x:f>IF(COUNTA(I17:L17)=0,"",ROUND(C17*I17+D17*J17+E17*K17+F17*L17,2))</x:f>
         <x:v>120</x:v>
       </x:c>
       <x:c r="N17" s="14">
@@ -2129,7 +2129,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="M18" s="13" t="n">
-        <x:f>IF(COUNTA(I18:L18)=0,"",C18*I18+D18*J18+E18*K18+F18*L18)</x:f>
+        <x:f>IF(COUNTA(I18:L18)=0,"",ROUND(C18*I18+D18*J18+E18*K18+F18*L18,2))</x:f>
         <x:v>220</x:v>
       </x:c>
       <x:c r="N18" s="14">
@@ -2178,7 +2178,7 @@
         <x:v>34</x:v>
       </x:c>
       <x:c r="M19" s="13" t="n">
-        <x:f>IF(COUNTA(I19:L19)=0,"",C19*I19+D19*J19+E19*K19+F19*L19)</x:f>
+        <x:f>IF(COUNTA(I19:L19)=0,"",ROUND(C19*I19+D19*J19+E19*K19+F19*L19,2))</x:f>
         <x:v>200</x:v>
       </x:c>
       <x:c r="N19" s="14">
@@ -2227,7 +2227,7 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="M20" s="13" t="n">
-        <x:f>IF(COUNTA(I20:L20)=0,"",C20*I20+D20*J20+E20*K20+F20*L20)</x:f>
+        <x:f>IF(COUNTA(I20:L20)=0,"",ROUND(C20*I20+D20*J20+E20*K20+F20*L20,2))</x:f>
         <x:v>184</x:v>
       </x:c>
       <x:c r="N20" s="14">
@@ -2276,7 +2276,7 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="M21" s="13" t="n">
-        <x:f>IF(COUNTA(I21:L21)=0,"",C21*I21+D21*J21+E21*K21+F21*L21)</x:f>
+        <x:f>IF(COUNTA(I21:L21)=0,"",ROUND(C21*I21+D21*J21+E21*K21+F21*L21,2))</x:f>
         <x:v>184</x:v>
       </x:c>
       <x:c r="N21" s="14">
@@ -2325,7 +2325,7 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="M22" s="13" t="n">
-        <x:f>IF(COUNTA(I22:L22)=0,"",C22*I22+D22*J22+E22*K22+F22*L22)</x:f>
+        <x:f>IF(COUNTA(I22:L22)=0,"",ROUND(C22*I22+D22*J22+E22*K22+F22*L22,2))</x:f>
         <x:v>184</x:v>
       </x:c>
       <x:c r="N22" s="14">
@@ -2374,7 +2374,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="M23" s="13" t="n">
-        <x:f>IF(COUNTA(I23:L23)=0,"",C23*I23+D23*J23+E23*K23+F23*L23)</x:f>
+        <x:f>IF(COUNTA(I23:L23)=0,"",ROUND(C23*I23+D23*J23+E23*K23+F23*L23,2))</x:f>
         <x:v>154</x:v>
       </x:c>
       <x:c r="N23" s="14">
@@ -2423,7 +2423,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="M24" s="13" t="n">
-        <x:f>IF(COUNTA(I24:L24)=0,"",C24*I24+D24*J24+E24*K24+F24*L24)</x:f>
+        <x:f>IF(COUNTA(I24:L24)=0,"",ROUND(C24*I24+D24*J24+E24*K24+F24*L24,2))</x:f>
         <x:v>146</x:v>
       </x:c>
       <x:c r="N24" s="14">
@@ -2472,7 +2472,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="M25" s="13" t="n">
-        <x:f>IF(COUNTA(I25:L25)=0,"",C25*I25+D25*J25+E25*K25+F25*L25)</x:f>
+        <x:f>IF(COUNTA(I25:L25)=0,"",ROUND(C25*I25+D25*J25+E25*K25+F25*L25,2))</x:f>
         <x:v>146</x:v>
       </x:c>
       <x:c r="N25" s="14">
@@ -2521,7 +2521,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="M26" s="13" t="n">
-        <x:f>IF(COUNTA(I26:L26)=0,"",C26*I26+D26*J26+E26*K26+F26*L26)</x:f>
+        <x:f>IF(COUNTA(I26:L26)=0,"",ROUND(C26*I26+D26*J26+E26*K26+F26*L26,2))</x:f>
         <x:v>146</x:v>
       </x:c>
       <x:c r="N26" s="14">
@@ -2570,7 +2570,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="M27" s="13" t="n">
-        <x:f>IF(COUNTA(I27:L27)=0,"",C27*I27+D27*J27+E27*K27+F27*L27)</x:f>
+        <x:f>IF(COUNTA(I27:L27)=0,"",ROUND(C27*I27+D27*J27+E27*K27+F27*L27,2))</x:f>
         <x:v>268</x:v>
       </x:c>
       <x:c r="N27" s="14">
@@ -2619,7 +2619,7 @@
         <x:v>34</x:v>
       </x:c>
       <x:c r="M28" s="13" t="n">
-        <x:f>IF(COUNTA(I28:L28)=0,"",C28*I28+D28*J28+E28*K28+F28*L28)</x:f>
+        <x:f>IF(COUNTA(I28:L28)=0,"",ROUND(C28*I28+D28*J28+E28*K28+F28*L28,2))</x:f>
         <x:v>240</x:v>
       </x:c>
       <x:c r="N28" s="14">
@@ -2668,7 +2668,7 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="M29" s="13" t="n">
-        <x:f>IF(COUNTA(I29:L29)=0,"",C29*I29+D29*J29+E29*K29+F29*L29)</x:f>
+        <x:f>IF(COUNTA(I29:L29)=0,"",ROUND(C29*I29+D29*J29+E29*K29+F29*L29,2))</x:f>
         <x:v>220</x:v>
       </x:c>
       <x:c r="N29" s="14">
@@ -2717,7 +2717,7 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="M30" s="13" t="n">
-        <x:f>IF(COUNTA(I30:L30)=0,"",C30*I30+D30*J30+E30*K30+F30*L30)</x:f>
+        <x:f>IF(COUNTA(I30:L30)=0,"",ROUND(C30*I30+D30*J30+E30*K30+F30*L30,2))</x:f>
         <x:v>220</x:v>
       </x:c>
       <x:c r="N30" s="14">
@@ -2766,7 +2766,7 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="M31" s="13" t="n">
-        <x:f>IF(COUNTA(I31:L31)=0,"",C31*I31+D31*J31+E31*K31+F31*L31)</x:f>
+        <x:f>IF(COUNTA(I31:L31)=0,"",ROUND(C31*I31+D31*J31+E31*K31+F31*L31,2))</x:f>
         <x:v>220</x:v>
       </x:c>
       <x:c r="N31" s="14">

</xml_diff>

<commit_message>
Use SKU keys for frame package pricing
</commit_message>
<xml_diff>
--- a/apps/moment-booth-fe/data/frame-package-pricing.xlsx
+++ b/apps/moment-booth-fe/data/frame-package-pricing.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Frame Pricing" sheetId="1" r:id="Rd3442a270afe42b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Frame Pricing" sheetId="1" r:id="Raaf58ca395ed4463"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -58,15 +58,15 @@
     <x:t xml:space="preserve">New Package Price (SGD)</x:t>
   </x:si>
   <x:si>
+    <x:t xml:space="preserve">Package guide</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Total frames</x:t>
+  </x:si>
+  <x:si>
     <x:t xml:space="preserve">Size breakdown</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Package guide</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Total frames</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Positioning</x:t>
   </x:si>
   <x:si>
@@ -85,19 +85,19 @@
     <x:t xml:space="preserve">White Rounded Border</x:t>
   </x:si>
   <x:si>
+    <x:t xml:space="preserve">8-piece package</x:t>
+  </x:si>
+  <x:si>
     <x:t xml:space="preserve">4 × 8", 2 × 10", 2 × 12"</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">8-piece package</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Silver Rounded Border</x:t>
   </x:si>
   <x:si>
+    <x:t xml:space="preserve">10-piece package</x:t>
+  </x:si>
+  <x:si>
     <x:t xml:space="preserve">6 × 8", 2 × 10", 2 × 12"</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">10-piece package</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Most Popular</x:t>
@@ -1389,17 +1389,17 @@
       <x:c r="O4" s="22" t="str">
         <x:v>Size note</x:v>
       </x:c>
-      <x:c r="P4" s="8" t="s">
+      <x:c r="P4" s="8" t="str">
+        <x:v>SKU</x:v>
+      </x:c>
+      <x:c r="Q4" s="8" t="s">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="Q4" s="8" t="s">
+      <x:c r="R4" t="s">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="R4" t="s">
+      <x:c r="S4" t="s">
         <x:v>18</x:v>
-      </x:c>
-      <x:c r="S4" t="s">
-        <x:v>16</x:v>
       </x:c>
       <x:c r="T4" t="s">
         <x:v>19</x:v>
@@ -1453,8 +1453,8 @@
       <x:c r="O5" s="15" t="str">
         <x:v>12" option applies to this frame type.</x:v>
       </x:c>
-      <x:c r="P5" s="16" t="s">
-        <x:v>23</x:v>
+      <x:c r="P5" s="16" t="str">
+        <x:v>6-piece-package-frameless-rounded-corner</x:v>
       </x:c>
       <x:c r="Q5" s="16" t="s">
         <x:v>20</x:v>
@@ -1517,17 +1517,17 @@
       <x:c r="O6" s="15" t="str">
         <x:v>12" option applies to this frame type.</x:v>
       </x:c>
-      <x:c r="P6" s="16" t="s">
+      <x:c r="P6" s="16" t="str">
+        <x:v>6-piece-package-white-rounded-border</x:v>
+      </x:c>
+      <x:c r="Q6" s="16" t="s">
         <x:v>25</x:v>
-      </x:c>
-      <x:c r="Q6" s="16" t="s">
-        <x:v>26</x:v>
       </x:c>
       <x:c r="R6">
         <x:v>8</x:v>
       </x:c>
       <x:c r="S6" t="s">
-        <x:v>25</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="T6" t="s">
         <x:v>21</x:v>
@@ -1581,17 +1581,17 @@
       <x:c r="O7" s="15" t="str">
         <x:v>12" option applies to this frame type.</x:v>
       </x:c>
-      <x:c r="P7" s="16" t="s">
+      <x:c r="P7" s="16" t="str">
+        <x:v>6-piece-package-silver-rounded-border</x:v>
+      </x:c>
+      <x:c r="Q7" s="17" t="s">
         <x:v>28</x:v>
-      </x:c>
-      <x:c r="Q7" s="17" t="s">
-        <x:v>29</x:v>
       </x:c>
       <x:c r="R7">
         <x:v>10</x:v>
       </x:c>
       <x:c r="S7" t="s">
-        <x:v>28</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="T7" t="s">
         <x:v>30</x:v>
@@ -1645,6 +1645,9 @@
       <x:c r="O8" s="18" t="str">
         <x:v>12" option applies to this frame type.</x:v>
       </x:c>
+      <x:c r="P8" t="str">
+        <x:v>6-piece-package-black-rounded-border</x:v>
+      </x:c>
     </x:row>
     <x:row r="9" ht="24" customHeight="1">
       <x:c r="A9" s="9" t="s">
@@ -1694,7 +1697,9 @@
       <x:c r="O9" s="19" t="str">
         <x:v>12" option applies to this frame type.</x:v>
       </x:c>
-      <x:c r="P9" s="20"/>
+      <x:c r="P9" s="20" t="str">
+        <x:v>6-piece-package-gold-square-corner</x:v>
+      </x:c>
       <x:c r="Q9" s="20" t="s">
         <x:v>33</x:v>
       </x:c>
@@ -1747,6 +1752,9 @@
       <x:c r="O10" s="18" t="str">
         <x:v>A4 replaces the 12" option for this frame type.</x:v>
       </x:c>
+      <x:c r="P10" t="str">
+        <x:v>6-piece-package-solid-wood-warm-walnut</x:v>
+      </x:c>
     </x:row>
     <x:row r="11" ht="24" customHeight="1">
       <x:c r="A11" s="9" t="s">
@@ -1796,6 +1804,9 @@
       <x:c r="O11" s="18" t="str">
         <x:v>A4 replaces the 12" option for this frame type.</x:v>
       </x:c>
+      <x:c r="P11" t="str">
+        <x:v>6-piece-package-fresh-light-wheat</x:v>
+      </x:c>
     </x:row>
     <x:row r="12" ht="24" customHeight="1">
       <x:c r="A12" s="9" t="s">
@@ -1845,6 +1856,9 @@
       <x:c r="O12" s="18" t="str">
         <x:v>A4 replaces the 12" option for this frame type.</x:v>
       </x:c>
+      <x:c r="P12" t="str">
+        <x:v>6-piece-package-roasted-tea</x:v>
+      </x:c>
     </x:row>
     <x:row r="13" ht="24" customHeight="1">
       <x:c r="A13" s="9" t="s">
@@ -1894,10 +1908,13 @@
       <x:c r="O13" s="18" t="str">
         <x:v>A4 replaces the 12" option for this frame type.</x:v>
       </x:c>
+      <x:c r="P13" t="str">
+        <x:v>6-piece-package-black-walnut</x:v>
+      </x:c>
     </x:row>
     <x:row r="14" ht="24" customHeight="1">
       <x:c r="A14" s="9" t="s">
-        <x:v>26</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="B14" s="9" t="s">
         <x:v>21</x:v>
@@ -1943,10 +1960,13 @@
       <x:c r="O14" s="18" t="str">
         <x:v>12" option applies to this frame type.</x:v>
       </x:c>
+      <x:c r="P14" t="str">
+        <x:v>8-piece-package-frameless-rounded-corner</x:v>
+      </x:c>
     </x:row>
     <x:row r="15" ht="24" customHeight="1">
       <x:c r="A15" s="9" t="s">
-        <x:v>26</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="B15" s="9" t="s">
         <x:v>21</x:v>
@@ -1992,10 +2012,13 @@
       <x:c r="O15" s="18" t="str">
         <x:v>12" option applies to this frame type.</x:v>
       </x:c>
+      <x:c r="P15" t="str">
+        <x:v>8-piece-package-white-rounded-border</x:v>
+      </x:c>
     </x:row>
     <x:row r="16" ht="24" customHeight="1">
       <x:c r="A16" s="9" t="s">
-        <x:v>26</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="B16" s="9" t="s">
         <x:v>21</x:v>
@@ -2041,10 +2064,13 @@
       <x:c r="O16" s="18" t="str">
         <x:v>12" option applies to this frame type.</x:v>
       </x:c>
+      <x:c r="P16" t="str">
+        <x:v>8-piece-package-silver-rounded-border</x:v>
+      </x:c>
     </x:row>
     <x:row r="17" ht="24" customHeight="1">
       <x:c r="A17" s="9" t="s">
-        <x:v>26</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="B17" s="9" t="s">
         <x:v>21</x:v>
@@ -2090,10 +2116,13 @@
       <x:c r="O17" s="18" t="str">
         <x:v>12" option applies to this frame type.</x:v>
       </x:c>
+      <x:c r="P17" t="str">
+        <x:v>8-piece-package-black-rounded-border</x:v>
+      </x:c>
     </x:row>
     <x:row r="18" ht="24" customHeight="1">
       <x:c r="A18" s="9" t="s">
-        <x:v>26</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="B18" s="9" t="s">
         <x:v>21</x:v>
@@ -2139,10 +2168,13 @@
       <x:c r="O18" s="18" t="str">
         <x:v>12" option applies to this frame type.</x:v>
       </x:c>
+      <x:c r="P18" t="str">
+        <x:v>8-piece-package-gold-square-corner</x:v>
+      </x:c>
     </x:row>
     <x:row r="19" ht="24" customHeight="1">
       <x:c r="A19" s="9" t="s">
-        <x:v>26</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="B19" s="9" t="s">
         <x:v>21</x:v>
@@ -2188,10 +2220,13 @@
       <x:c r="O19" s="18" t="str">
         <x:v>A4 replaces the 12" option for this frame type.</x:v>
       </x:c>
+      <x:c r="P19" t="str">
+        <x:v>8-piece-package-solid-wood-warm-walnut</x:v>
+      </x:c>
     </x:row>
     <x:row r="20" ht="24" customHeight="1">
       <x:c r="A20" s="9" t="s">
-        <x:v>26</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="B20" s="9" t="s">
         <x:v>21</x:v>
@@ -2237,10 +2272,13 @@
       <x:c r="O20" s="18" t="str">
         <x:v>A4 replaces the 12" option for this frame type.</x:v>
       </x:c>
+      <x:c r="P20" t="str">
+        <x:v>8-piece-package-fresh-light-wheat</x:v>
+      </x:c>
     </x:row>
     <x:row r="21" ht="24" customHeight="1">
       <x:c r="A21" s="9" t="s">
-        <x:v>26</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="B21" s="9" t="s">
         <x:v>21</x:v>
@@ -2286,10 +2324,13 @@
       <x:c r="O21" s="18" t="str">
         <x:v>A4 replaces the 12" option for this frame type.</x:v>
       </x:c>
+      <x:c r="P21" t="str">
+        <x:v>8-piece-package-roasted-tea</x:v>
+      </x:c>
     </x:row>
     <x:row r="22" ht="24" customHeight="1">
       <x:c r="A22" s="9" t="s">
-        <x:v>26</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="B22" s="9" t="s">
         <x:v>21</x:v>
@@ -2335,10 +2376,13 @@
       <x:c r="O22" s="18" t="str">
         <x:v>A4 replaces the 12" option for this frame type.</x:v>
       </x:c>
+      <x:c r="P22" t="str">
+        <x:v>8-piece-package-black-walnut</x:v>
+      </x:c>
     </x:row>
     <x:row r="23" ht="24" customHeight="1">
       <x:c r="A23" s="9" t="s">
-        <x:v>29</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="B23" s="21" t="s">
         <x:v>30</x:v>
@@ -2384,10 +2428,13 @@
       <x:c r="O23" s="18" t="str">
         <x:v>12" option applies to this frame type.</x:v>
       </x:c>
+      <x:c r="P23" t="str">
+        <x:v>10-piece-package-frameless-rounded-corner</x:v>
+      </x:c>
     </x:row>
     <x:row r="24" ht="24" customHeight="1">
       <x:c r="A24" s="9" t="s">
-        <x:v>29</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="B24" s="21" t="s">
         <x:v>30</x:v>
@@ -2433,10 +2480,13 @@
       <x:c r="O24" s="18" t="str">
         <x:v>12" option applies to this frame type.</x:v>
       </x:c>
+      <x:c r="P24" t="str">
+        <x:v>10-piece-package-white-rounded-border</x:v>
+      </x:c>
     </x:row>
     <x:row r="25" ht="24" customHeight="1">
       <x:c r="A25" s="9" t="s">
-        <x:v>29</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="B25" s="21" t="s">
         <x:v>30</x:v>
@@ -2482,10 +2532,13 @@
       <x:c r="O25" s="18" t="str">
         <x:v>12" option applies to this frame type.</x:v>
       </x:c>
+      <x:c r="P25" t="str">
+        <x:v>10-piece-package-silver-rounded-border</x:v>
+      </x:c>
     </x:row>
     <x:row r="26" ht="24" customHeight="1">
       <x:c r="A26" s="9" t="s">
-        <x:v>29</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="B26" s="21" t="s">
         <x:v>30</x:v>
@@ -2531,10 +2584,13 @@
       <x:c r="O26" s="18" t="str">
         <x:v>12" option applies to this frame type.</x:v>
       </x:c>
+      <x:c r="P26" t="str">
+        <x:v>10-piece-package-black-rounded-border</x:v>
+      </x:c>
     </x:row>
     <x:row r="27" ht="24" customHeight="1">
       <x:c r="A27" s="9" t="s">
-        <x:v>29</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="B27" s="21" t="s">
         <x:v>30</x:v>
@@ -2580,10 +2636,13 @@
       <x:c r="O27" s="18" t="str">
         <x:v>12" option applies to this frame type.</x:v>
       </x:c>
+      <x:c r="P27" t="str">
+        <x:v>10-piece-package-gold-square-corner</x:v>
+      </x:c>
     </x:row>
     <x:row r="28" ht="24" customHeight="1">
       <x:c r="A28" s="9" t="s">
-        <x:v>29</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="B28" s="21" t="s">
         <x:v>30</x:v>
@@ -2629,10 +2688,13 @@
       <x:c r="O28" s="18" t="str">
         <x:v>A4 replaces the 12" option for this frame type.</x:v>
       </x:c>
+      <x:c r="P28" t="str">
+        <x:v>10-piece-package-solid-wood-warm-walnut</x:v>
+      </x:c>
     </x:row>
     <x:row r="29" ht="24" customHeight="1">
       <x:c r="A29" s="9" t="s">
-        <x:v>29</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="B29" s="21" t="s">
         <x:v>30</x:v>
@@ -2678,10 +2740,13 @@
       <x:c r="O29" s="18" t="str">
         <x:v>A4 replaces the 12" option for this frame type.</x:v>
       </x:c>
+      <x:c r="P29" t="str">
+        <x:v>10-piece-package-fresh-light-wheat</x:v>
+      </x:c>
     </x:row>
     <x:row r="30" ht="24" customHeight="1">
       <x:c r="A30" s="9" t="s">
-        <x:v>29</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="B30" s="21" t="s">
         <x:v>30</x:v>
@@ -2727,10 +2792,13 @@
       <x:c r="O30" s="18" t="str">
         <x:v>A4 replaces the 12" option for this frame type.</x:v>
       </x:c>
+      <x:c r="P30" t="str">
+        <x:v>10-piece-package-roasted-tea</x:v>
+      </x:c>
     </x:row>
     <x:row r="31" ht="24" customHeight="1">
       <x:c r="A31" s="9" t="s">
-        <x:v>29</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="B31" s="21" t="s">
         <x:v>30</x:v>
@@ -2775,6 +2843,9 @@
       </x:c>
       <x:c r="O31" s="18" t="str">
         <x:v>A4 replaces the 12" option for this frame type.</x:v>
+      </x:c>
+      <x:c r="P31" t="str">
+        <x:v>10-piece-package-black-walnut</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Set frame package prices to ninety percent
</commit_message>
<xml_diff>
--- a/apps/moment-booth-fe/data/frame-package-pricing.xlsx
+++ b/apps/moment-booth-fe/data/frame-package-pricing.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Frame Pricing" sheetId="1" r:id="Raaf58ca395ed4463"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Frame Pricing" sheetId="1" r:id="R4725229aac734e70"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1447,8 +1447,8 @@
         <x:v>102</x:v>
       </x:c>
       <x:c r="N5" s="14" t="n">
-        <x:f>M5*0.8</x:f>
-        <x:v>81.60000000000001</x:v>
+        <x:f>ROUND(M5*0.9,2)</x:f>
+        <x:v>91.8</x:v>
       </x:c>
       <x:c r="O5" s="15" t="str">
         <x:v>12" option applies to this frame type.</x:v>
@@ -1511,8 +1511,8 @@
         <x:v>94</x:v>
       </x:c>
       <x:c r="N6" s="14" t="n">
-        <x:f t="shared" ref="N6:N31" si="1">M6*0.8</x:f>
-        <x:v>75.2</x:v>
+        <x:f t="shared" ref="N6:N31" si="1">ROUND(M6*0.9,2)</x:f>
+        <x:v>84.6</x:v>
       </x:c>
       <x:c r="O6" s="15" t="str">
         <x:v>12" option applies to this frame type.</x:v>
@@ -1574,9 +1574,9 @@
         <x:f>IF(COUNTA(I7:L7)=0,"",ROUND(C7*I7+D7*J7+E7*K7+F7*L7,2))</x:f>
         <x:v>94</x:v>
       </x:c>
-      <x:c r="N7" s="14">
-        <x:f t="shared" si="1"/>
-        <x:v>75.2</x:v>
+      <x:c r="N7" s="14" t="n">
+        <x:f t="shared" si="1">ROUND(M7*0.9,2)</x:f>
+        <x:v>84.6</x:v>
       </x:c>
       <x:c r="O7" s="15" t="str">
         <x:v>12" option applies to this frame type.</x:v>
@@ -1638,9 +1638,9 @@
         <x:f>IF(COUNTA(I8:L8)=0,"",ROUND(C8*I8+D8*J8+E8*K8+F8*L8,2))</x:f>
         <x:v>94</x:v>
       </x:c>
-      <x:c r="N8" s="14">
-        <x:f t="shared" si="1"/>
-        <x:v>75.2</x:v>
+      <x:c r="N8" s="14" t="n">
+        <x:f t="shared" si="1">ROUND(M8*0.9,2)</x:f>
+        <x:v>84.6</x:v>
       </x:c>
       <x:c r="O8" s="18" t="str">
         <x:v>12" option applies to this frame type.</x:v>
@@ -1690,9 +1690,9 @@
         <x:f>IF(COUNTA(I9:L9)=0,"",ROUND(C9*I9+D9*J9+E9*K9+F9*L9,2))</x:f>
         <x:v>172</x:v>
       </x:c>
-      <x:c r="N9" s="14">
-        <x:f t="shared" si="1"/>
-        <x:v>137.6</x:v>
+      <x:c r="N9" s="14" t="n">
+        <x:f t="shared" si="1">ROUND(M9*0.9,2)</x:f>
+        <x:v>154.8</x:v>
       </x:c>
       <x:c r="O9" s="19" t="str">
         <x:v>12" option applies to this frame type.</x:v>
@@ -1745,9 +1745,9 @@
         <x:f>IF(COUNTA(I10:L10)=0,"",ROUND(C10*I10+D10*J10+E10*K10+F10*L10,2))</x:f>
         <x:v>160</x:v>
       </x:c>
-      <x:c r="N10" s="14">
-        <x:f t="shared" si="1"/>
-        <x:v>73.6</x:v>
+      <x:c r="N10" s="14" t="n">
+        <x:f t="shared" si="1">ROUND(M10*0.9,2)</x:f>
+        <x:v>144</x:v>
       </x:c>
       <x:c r="O10" s="18" t="str">
         <x:v>A4 replaces the 12" option for this frame type.</x:v>
@@ -1797,9 +1797,9 @@
         <x:f>IF(COUNTA(I11:L11)=0,"",ROUND(C11*I11+D11*J11+E11*K11+F11*L11,2))</x:f>
         <x:v>148</x:v>
       </x:c>
-      <x:c r="N11" s="14">
-        <x:f t="shared" si="1"/>
-        <x:v>70.4</x:v>
+      <x:c r="N11" s="14" t="n">
+        <x:f t="shared" si="1">ROUND(M11*0.9,2)</x:f>
+        <x:v>133.2</x:v>
       </x:c>
       <x:c r="O11" s="18" t="str">
         <x:v>A4 replaces the 12" option for this frame type.</x:v>
@@ -1849,9 +1849,9 @@
         <x:f>IF(COUNTA(I12:L12)=0,"",ROUND(C12*I12+D12*J12+E12*K12+F12*L12,2))</x:f>
         <x:v>148</x:v>
       </x:c>
-      <x:c r="N12" s="14">
-        <x:f t="shared" si="1"/>
-        <x:v>70.4</x:v>
+      <x:c r="N12" s="14" t="n">
+        <x:f t="shared" si="1">ROUND(M12*0.9,2)</x:f>
+        <x:v>133.2</x:v>
       </x:c>
       <x:c r="O12" s="18" t="str">
         <x:v>A4 replaces the 12" option for this frame type.</x:v>
@@ -1901,9 +1901,9 @@
         <x:f>IF(COUNTA(I13:L13)=0,"",ROUND(C13*I13+D13*J13+E13*K13+F13*L13,2))</x:f>
         <x:v>148</x:v>
       </x:c>
-      <x:c r="N13" s="14">
-        <x:f t="shared" si="1"/>
-        <x:v>70.4</x:v>
+      <x:c r="N13" s="14" t="n">
+        <x:f t="shared" si="1">ROUND(M13*0.9,2)</x:f>
+        <x:v>133.2</x:v>
       </x:c>
       <x:c r="O13" s="18" t="str">
         <x:v>A4 replaces the 12" option for this frame type.</x:v>
@@ -1953,9 +1953,9 @@
         <x:f>IF(COUNTA(I14:L14)=0,"",ROUND(C14*I14+D14*J14+E14*K14+F14*L14,2))</x:f>
         <x:v>128</x:v>
       </x:c>
-      <x:c r="N14" s="14">
-        <x:f t="shared" si="1"/>
-        <x:v>102.4</x:v>
+      <x:c r="N14" s="14" t="n">
+        <x:f t="shared" si="1">ROUND(M14*0.9,2)</x:f>
+        <x:v>115.2</x:v>
       </x:c>
       <x:c r="O14" s="18" t="str">
         <x:v>12" option applies to this frame type.</x:v>
@@ -2005,9 +2005,9 @@
         <x:f>IF(COUNTA(I15:L15)=0,"",ROUND(C15*I15+D15*J15+E15*K15+F15*L15,2))</x:f>
         <x:v>120</x:v>
       </x:c>
-      <x:c r="N15" s="14">
-        <x:f t="shared" si="1"/>
-        <x:v>96</x:v>
+      <x:c r="N15" s="14" t="n">
+        <x:f t="shared" si="1">ROUND(M15*0.9,2)</x:f>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="O15" s="18" t="str">
         <x:v>12" option applies to this frame type.</x:v>
@@ -2057,9 +2057,9 @@
         <x:f>IF(COUNTA(I16:L16)=0,"",ROUND(C16*I16+D16*J16+E16*K16+F16*L16,2))</x:f>
         <x:v>120</x:v>
       </x:c>
-      <x:c r="N16" s="14">
-        <x:f t="shared" si="1"/>
-        <x:v>96</x:v>
+      <x:c r="N16" s="14" t="n">
+        <x:f t="shared" si="1">ROUND(M16*0.9,2)</x:f>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="O16" s="18" t="str">
         <x:v>12" option applies to this frame type.</x:v>
@@ -2109,9 +2109,9 @@
         <x:f>IF(COUNTA(I17:L17)=0,"",ROUND(C17*I17+D17*J17+E17*K17+F17*L17,2))</x:f>
         <x:v>120</x:v>
       </x:c>
-      <x:c r="N17" s="14">
-        <x:f t="shared" si="1"/>
-        <x:v>96</x:v>
+      <x:c r="N17" s="14" t="n">
+        <x:f t="shared" si="1">ROUND(M17*0.9,2)</x:f>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="O17" s="18" t="str">
         <x:v>12" option applies to this frame type.</x:v>
@@ -2161,9 +2161,9 @@
         <x:f>IF(COUNTA(I18:L18)=0,"",ROUND(C18*I18+D18*J18+E18*K18+F18*L18,2))</x:f>
         <x:v>220</x:v>
       </x:c>
-      <x:c r="N18" s="14">
-        <x:f t="shared" si="1"/>
-        <x:v>176</x:v>
+      <x:c r="N18" s="14" t="n">
+        <x:f t="shared" si="1">ROUND(M18*0.9,2)</x:f>
+        <x:v>198</x:v>
       </x:c>
       <x:c r="O18" s="18" t="str">
         <x:v>12" option applies to this frame type.</x:v>
@@ -2213,9 +2213,9 @@
         <x:f>IF(COUNTA(I19:L19)=0,"",ROUND(C19*I19+D19*J19+E19*K19+F19*L19,2))</x:f>
         <x:v>200</x:v>
       </x:c>
-      <x:c r="N19" s="14">
-        <x:f t="shared" si="1"/>
-        <x:v>105.6</x:v>
+      <x:c r="N19" s="14" t="n">
+        <x:f t="shared" si="1">ROUND(M19*0.9,2)</x:f>
+        <x:v>180</x:v>
       </x:c>
       <x:c r="O19" s="18" t="str">
         <x:v>A4 replaces the 12" option for this frame type.</x:v>
@@ -2265,9 +2265,9 @@
         <x:f>IF(COUNTA(I20:L20)=0,"",ROUND(C20*I20+D20*J20+E20*K20+F20*L20,2))</x:f>
         <x:v>184</x:v>
       </x:c>
-      <x:c r="N20" s="14">
-        <x:f t="shared" si="1"/>
-        <x:v>99.2</x:v>
+      <x:c r="N20" s="14" t="n">
+        <x:f t="shared" si="1">ROUND(M20*0.9,2)</x:f>
+        <x:v>165.6</x:v>
       </x:c>
       <x:c r="O20" s="18" t="str">
         <x:v>A4 replaces the 12" option for this frame type.</x:v>
@@ -2317,9 +2317,9 @@
         <x:f>IF(COUNTA(I21:L21)=0,"",ROUND(C21*I21+D21*J21+E21*K21+F21*L21,2))</x:f>
         <x:v>184</x:v>
       </x:c>
-      <x:c r="N21" s="14">
-        <x:f t="shared" si="1"/>
-        <x:v>99.2</x:v>
+      <x:c r="N21" s="14" t="n">
+        <x:f t="shared" si="1">ROUND(M21*0.9,2)</x:f>
+        <x:v>165.6</x:v>
       </x:c>
       <x:c r="O21" s="18" t="str">
         <x:v>A4 replaces the 12" option for this frame type.</x:v>
@@ -2369,9 +2369,9 @@
         <x:f>IF(COUNTA(I22:L22)=0,"",ROUND(C22*I22+D22*J22+E22*K22+F22*L22,2))</x:f>
         <x:v>184</x:v>
       </x:c>
-      <x:c r="N22" s="14">
-        <x:f t="shared" si="1"/>
-        <x:v>99.2</x:v>
+      <x:c r="N22" s="14" t="n">
+        <x:f t="shared" si="1">ROUND(M22*0.9,2)</x:f>
+        <x:v>165.6</x:v>
       </x:c>
       <x:c r="O22" s="18" t="str">
         <x:v>A4 replaces the 12" option for this frame type.</x:v>
@@ -2421,9 +2421,9 @@
         <x:f>IF(COUNTA(I23:L23)=0,"",ROUND(C23*I23+D23*J23+E23*K23+F23*L23,2))</x:f>
         <x:v>154</x:v>
       </x:c>
-      <x:c r="N23" s="14">
-        <x:f t="shared" si="1"/>
-        <x:v>123.2</x:v>
+      <x:c r="N23" s="14" t="n">
+        <x:f t="shared" si="1">ROUND(M23*0.9,2)</x:f>
+        <x:v>138.6</x:v>
       </x:c>
       <x:c r="O23" s="18" t="str">
         <x:v>12" option applies to this frame type.</x:v>
@@ -2473,9 +2473,9 @@
         <x:f>IF(COUNTA(I24:L24)=0,"",ROUND(C24*I24+D24*J24+E24*K24+F24*L24,2))</x:f>
         <x:v>146</x:v>
       </x:c>
-      <x:c r="N24" s="14">
-        <x:f t="shared" si="1"/>
-        <x:v>116.8</x:v>
+      <x:c r="N24" s="14" t="n">
+        <x:f t="shared" si="1">ROUND(M24*0.9,2)</x:f>
+        <x:v>131.4</x:v>
       </x:c>
       <x:c r="O24" s="18" t="str">
         <x:v>12" option applies to this frame type.</x:v>
@@ -2525,9 +2525,9 @@
         <x:f>IF(COUNTA(I25:L25)=0,"",ROUND(C25*I25+D25*J25+E25*K25+F25*L25,2))</x:f>
         <x:v>146</x:v>
       </x:c>
-      <x:c r="N25" s="14">
-        <x:f t="shared" si="1"/>
-        <x:v>116.8</x:v>
+      <x:c r="N25" s="14" t="n">
+        <x:f t="shared" si="1">ROUND(M25*0.9,2)</x:f>
+        <x:v>131.4</x:v>
       </x:c>
       <x:c r="O25" s="18" t="str">
         <x:v>12" option applies to this frame type.</x:v>
@@ -2577,9 +2577,9 @@
         <x:f>IF(COUNTA(I26:L26)=0,"",ROUND(C26*I26+D26*J26+E26*K26+F26*L26,2))</x:f>
         <x:v>146</x:v>
       </x:c>
-      <x:c r="N26" s="14">
-        <x:f t="shared" si="1"/>
-        <x:v>116.8</x:v>
+      <x:c r="N26" s="14" t="n">
+        <x:f t="shared" si="1">ROUND(M26*0.9,2)</x:f>
+        <x:v>131.4</x:v>
       </x:c>
       <x:c r="O26" s="18" t="str">
         <x:v>12" option applies to this frame type.</x:v>
@@ -2629,9 +2629,9 @@
         <x:f>IF(COUNTA(I27:L27)=0,"",ROUND(C27*I27+D27*J27+E27*K27+F27*L27,2))</x:f>
         <x:v>268</x:v>
       </x:c>
-      <x:c r="N27" s="14">
-        <x:f t="shared" si="1"/>
-        <x:v>214.4</x:v>
+      <x:c r="N27" s="14" t="n">
+        <x:f t="shared" si="1">ROUND(M27*0.9,2)</x:f>
+        <x:v>241.2</x:v>
       </x:c>
       <x:c r="O27" s="18" t="str">
         <x:v>12" option applies to this frame type.</x:v>
@@ -2681,9 +2681,9 @@
         <x:f>IF(COUNTA(I28:L28)=0,"",ROUND(C28*I28+D28*J28+E28*K28+F28*L28,2))</x:f>
         <x:v>240</x:v>
       </x:c>
-      <x:c r="N28" s="14">
-        <x:f t="shared" si="1"/>
-        <x:v>137.6</x:v>
+      <x:c r="N28" s="14" t="n">
+        <x:f t="shared" si="1">ROUND(M28*0.9,2)</x:f>
+        <x:v>216</x:v>
       </x:c>
       <x:c r="O28" s="18" t="str">
         <x:v>A4 replaces the 12" option for this frame type.</x:v>
@@ -2733,9 +2733,9 @@
         <x:f>IF(COUNTA(I29:L29)=0,"",ROUND(C29*I29+D29*J29+E29*K29+F29*L29,2))</x:f>
         <x:v>220</x:v>
       </x:c>
-      <x:c r="N29" s="14">
-        <x:f t="shared" si="1"/>
-        <x:v>128</x:v>
+      <x:c r="N29" s="14" t="n">
+        <x:f t="shared" si="1">ROUND(M29*0.9,2)</x:f>
+        <x:v>198</x:v>
       </x:c>
       <x:c r="O29" s="18" t="str">
         <x:v>A4 replaces the 12" option for this frame type.</x:v>
@@ -2785,9 +2785,9 @@
         <x:f>IF(COUNTA(I30:L30)=0,"",ROUND(C30*I30+D30*J30+E30*K30+F30*L30,2))</x:f>
         <x:v>220</x:v>
       </x:c>
-      <x:c r="N30" s="14">
-        <x:f t="shared" si="1"/>
-        <x:v>128</x:v>
+      <x:c r="N30" s="14" t="n">
+        <x:f t="shared" si="1">ROUND(M30*0.9,2)</x:f>
+        <x:v>198</x:v>
       </x:c>
       <x:c r="O30" s="18" t="str">
         <x:v>A4 replaces the 12" option for this frame type.</x:v>
@@ -2837,9 +2837,9 @@
         <x:f>IF(COUNTA(I31:L31)=0,"",ROUND(C31*I31+D31*J31+E31*K31+F31*L31,2))</x:f>
         <x:v>220</x:v>
       </x:c>
-      <x:c r="N31" s="14">
-        <x:f t="shared" si="1"/>
-        <x:v>128</x:v>
+      <x:c r="N31" s="14" t="n">
+        <x:f t="shared" si="1">ROUND(M31*0.9,2)</x:f>
+        <x:v>198</x:v>
       </x:c>
       <x:c r="O31" s="18" t="str">
         <x:v>A4 replaces the 12" option for this frame type.</x:v>

</xml_diff>